<commit_message>
Add final project deliverables and reports
Add final deliverables and generated outputs for multiple coursework projects. Includes TrabajoFinal artifacts (build_report.py, final notebook/docx/pdf, output CSVs and kmeans image) and saves notebook execution outputs. Adds Topicos-Selectos activity 9 deliverables and helper scripts (analyze.py, explore.py, generate_report.py) plus SKU analysis spreadsheet. Also updates small text/docx changes in programming and activity folders. These changes primarily add generated reports and deliverable files.
</commit_message>
<xml_diff>
--- a/2do-semestre/topicos-selectos-i/tareas/actividades/actividad-9/sku_analysis_output.xlsx
+++ b/2do-semestre/topicos-selectos-i/tareas/actividades/actividad-9/sku_analysis_output.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="39">
   <si>
     <t>ITEM</t>
   </si>
@@ -64,16 +64,16 @@
     <t>LED06/10W.</t>
   </si>
   <si>
+    <t>REFLED/300W</t>
+  </si>
+  <si>
     <t>SUBSOL/60W</t>
   </si>
   <si>
-    <t>LED06/10W3</t>
-  </si>
-  <si>
-    <t>ADAPTADOR/E40</t>
-  </si>
-  <si>
-    <t>LRD/9W</t>
+    <t>REFLED/200W</t>
+  </si>
+  <si>
+    <t>T-SUBFOT/100W-A</t>
   </si>
   <si>
     <t>B</t>
@@ -85,15 +85,15 @@
     <t>GROWING</t>
   </si>
   <si>
+    <t>DECLINING</t>
+  </si>
+  <si>
     <t>STABLE</t>
   </si>
   <si>
     <t>STRONG GROWTH</t>
   </si>
   <si>
-    <t>DECLINING</t>
-  </si>
-  <si>
     <t>CRITICAL</t>
   </si>
   <si>
@@ -103,37 +103,34 @@
     <t>MEDIUM</t>
   </si>
   <si>
-    <t>LOW</t>
-  </si>
-  <si>
     <t>Compra inmediata de 578,100 pzas (2.0 meses). Stock en mano: 0.73 meses. Stockout en 22 días (lead time: 120 días). Activar booking y anticipo urgente.</t>
   </si>
   <si>
+    <t>Compra inmediata de 520 pzas (1.5 meses). Stock en mano: 0.22 meses. Stockout en 7 días (lead time: 120 días). Activar booking y anticipo urgente.</t>
+  </si>
+  <si>
     <t>Compra inmediata de 2,250 pzas (2.0 meses). Stock en mano: 1.48 meses. Stockout en 44 días (lead time: 120 días). Activar booking y anticipo urgente.</t>
   </si>
   <si>
-    <t>Compra inmediata de 26,160 pzas (2.0 meses). Stock en mano: 0.03 meses. Stockout en 1 días (lead time: 120 días). Activar booking y anticipo urgente.</t>
-  </si>
-  <si>
-    <t>Compra inmediata de 500 pzas (1.9 meses). Stock en mano: 1.74 meses. Stockout en 52 días (lead time: 120 días). Activar booking y anticipo urgente.</t>
-  </si>
-  <si>
-    <t>Compra inmediata de 810 pzas (0.9 meses). Stock en mano: 1.17 meses. Stockout en 35 días (lead time: 120 días). Activar booking y anticipo urgente.</t>
+    <t>Compra inmediata de 1,960 pzas (1.3 meses). Stock en mano: 1.56 meses. Stockout en 47 días (lead time: 120 días). Activar booking y anticipo urgente.</t>
+  </si>
+  <si>
+    <t>Compra inmediata de 0 pzas (0.0 meses). Stock en mano: 0.87 meses. Stockout en 26 días (lead time: 120 días). Activar booking y anticipo urgente.</t>
   </si>
   <si>
     <t>Comprar urgentemente 578,100 piezas (~2.0 meses) y acelerar booking inmediato; stock actual de 210,412 piezas solo cubre 0.7 meses vs forecast mensual de 245,770. SKU B con tendencia GROWING. Riesgo: stockout en ~22 días.</t>
   </si>
   <si>
+    <t>Comprar urgentemente 520 piezas (~1.5 meses) y acelerar booking inmediato; stock actual de 56 piezas solo cubre 0.2 meses vs forecast mensual de 518. SKU B con tendencia DECLINING. Riesgo: stockout en ~7 días.</t>
+  </si>
+  <si>
     <t>Comprar urgentemente 2,250 piezas (~2.0 meses) y acelerar booking inmediato; stock actual de 1,672 piezas solo cubre 1.5 meses vs forecast mensual de 1,624. SKU A con tendencia STABLE. Riesgo: stockout en ~44 días.</t>
   </si>
   <si>
-    <t>Comprar urgentemente 26,160 piezas (~2.0 meses) y acelerar booking inmediato; stock actual de 329 piezas solo cubre 0.0 meses vs forecast mensual de 0. SKU B con tendencia STABLE. Riesgo: stockout en ~1 días.</t>
-  </si>
-  <si>
-    <t>Comprar normal 500 piezas para sostener cobertura objetivo de 1.9 meses; el SKU mantiene 1.7 meses en stock y 1.7 meses considerando supply chain total. Monitorear tendencia STRONG GROWTH.</t>
-  </si>
-  <si>
-    <t>Comprar urgentemente 810 piezas (~0.9 meses) y acelerar booking inmediato; stock actual de 839 piezas solo cubre 1.2 meses vs forecast mensual de 0. SKU B con tendencia DECLINING. Riesgo: stockout en ~35 días.</t>
+    <t>Comprar normal 1,960 piezas para sostener cobertura objetivo de 1.3 meses; el SKU mantiene 1.6 meses en stock y 4.8 meses considerando supply chain total. Monitorear tendencia DECLINING.</t>
+  </si>
+  <si>
+    <t>Acelerar booking de 2,360 piezas y priorizar carga marítima; la cobertura total es de 7.1 meses y existe atraso operativo en supply chain. Riesgo: retraso logístico.</t>
   </si>
 </sst>
 </file>
@@ -582,10 +579,10 @@
         <v>26</v>
       </c>
       <c r="N2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="O2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="3" spans="1:15">
@@ -593,7 +590,7 @@
         <v>16</v>
       </c>
       <c r="B3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C3" t="s">
         <v>23</v>
@@ -602,37 +599,37 @@
         <v>27</v>
       </c>
       <c r="E3">
-        <v>1.48</v>
+        <v>0.22</v>
       </c>
       <c r="F3">
-        <v>2.097690941385435</v>
+        <v>2.138461538461538</v>
       </c>
       <c r="G3">
-        <v>3.58</v>
+        <v>2.36</v>
       </c>
       <c r="H3">
-        <v>44.4</v>
+        <v>6.6</v>
       </c>
       <c r="I3">
-        <v>2250</v>
+        <v>520</v>
       </c>
       <c r="J3">
-        <v>2</v>
+        <v>1.5</v>
       </c>
       <c r="K3">
-        <v>-0.5921572706469732</v>
+        <v>-0.6370272063702721</v>
       </c>
       <c r="L3">
-        <v>30</v>
+        <v>12</v>
       </c>
       <c r="M3" t="s">
         <v>26</v>
       </c>
       <c r="N3" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="O3" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="4" spans="1:15">
@@ -640,46 +637,46 @@
         <v>17</v>
       </c>
       <c r="B4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D4" t="s">
         <v>27</v>
       </c>
       <c r="E4">
-        <v>0.03</v>
+        <v>1.48</v>
       </c>
       <c r="F4">
-        <v>0.3924554288774963</v>
+        <v>2.097690941385435</v>
       </c>
       <c r="G4">
-        <v>0.42</v>
+        <v>3.58</v>
       </c>
       <c r="H4">
-        <v>0.8999999999999999</v>
+        <v>44.4</v>
       </c>
       <c r="I4">
-        <v>26160</v>
+        <v>2250</v>
       </c>
       <c r="J4">
         <v>2</v>
       </c>
       <c r="K4">
-        <v>-0.2638652804680397</v>
+        <v>-0.5921572706469732</v>
       </c>
       <c r="L4">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="M4" t="s">
         <v>26</v>
       </c>
       <c r="N4" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="O4" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="5" spans="1:15">
@@ -690,43 +687,43 @@
         <v>20</v>
       </c>
       <c r="C5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D5" t="s">
         <v>28</v>
       </c>
       <c r="E5">
-        <v>1.74</v>
+        <v>1.56</v>
       </c>
       <c r="F5">
-        <v>1.740601503759398</v>
+        <v>4.758222222222222</v>
       </c>
       <c r="G5">
-        <v>3.48</v>
+        <v>6.32</v>
       </c>
       <c r="H5">
-        <v>52.2</v>
+        <v>46.8</v>
       </c>
       <c r="I5">
-        <v>500</v>
+        <v>1960</v>
       </c>
       <c r="J5">
-        <v>1.9</v>
+        <v>1.3</v>
       </c>
       <c r="K5">
-        <v>-0.07199999999999999</v>
+        <v>-0.6034297075635822</v>
       </c>
       <c r="L5">
-        <v>56</v>
+        <v>25</v>
       </c>
       <c r="M5" t="s">
         <v>26</v>
       </c>
       <c r="N5" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="O5" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="6" spans="1:15">
@@ -734,46 +731,40 @@
         <v>19</v>
       </c>
       <c r="B6" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C6" t="s">
         <v>25</v>
       </c>
       <c r="D6" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E6">
-        <v>1.17</v>
+        <v>0.87</v>
       </c>
       <c r="F6">
-        <v>5.369230769230769</v>
+        <v>7.116768499660557</v>
       </c>
       <c r="G6">
-        <v>6.54</v>
+        <v>7.99</v>
       </c>
       <c r="H6">
-        <v>35.09999999999999</v>
-      </c>
-      <c r="I6">
-        <v>810</v>
-      </c>
-      <c r="J6">
-        <v>0.9</v>
+        <v>26.1</v>
       </c>
       <c r="K6">
-        <v>-0.5675301288267073</v>
+        <v>-0.0728887807252372</v>
       </c>
       <c r="L6">
-        <v>8</v>
+        <v>76</v>
       </c>
       <c r="M6" t="s">
         <v>26</v>
       </c>
       <c r="N6" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="O6" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
   </sheetData>

</xml_diff>